<commit_message>
refactor(PDG-61): run post-normalization rules in sheet row order
Drop the priority-column sort in PostNormalizationEngine so rules run top-to-bottom as written, and remove the now-unused priority column from postNormalization.xlsx and mediaPostNormalization.xlsx.

postNormalization.xlsx also carries the defensive Identifiers[].IssuedDate/ExpiryDate DATE_NORMALIZATION row - bundled here because it is a single binary file.
</commit_message>
<xml_diff>
--- a/data/rules/mediaPostNormalization.xlsx
+++ b/data/rules/mediaPostNormalization.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE4466C7-7EA7-414C-B7D3-4EE4C2BC644D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD79B697-87DE-4F73-BE98-477C14218035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1590" yWindow="1750" windowWidth="12060" windowHeight="8320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
-  <si>
-    <t>priority</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>rule_type</t>
   </si>
@@ -322,18 +319,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="38" customWidth="1"/>
+    <col min="1" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="16" customHeight="1">
+    <row r="1" spans="1:6" ht="16" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -352,50 +348,38 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="2" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="2">
-        <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="2">
-        <v>100</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
+    <row r="3" spans="1:6">
+      <c r="A3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7">
-      <c r="A4">
-        <v>10</v>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>9</v>
       </c>
       <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(PDG-88): decode HTML entities in media titles and links
SANITIZE_HTML now also cleans a single nested field (Content.Title), not only array leaves. New post-normalization rows decode &amp; in Attachments[].URL and URLs[].URL before deduplication, and &#8217; etc. in titles, for every media source.
</commit_message>
<xml_diff>
--- a/data/rules/mediaPostNormalization.xlsx
+++ b/data/rules/mediaPostNormalization.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD79B697-87DE-4F73-BE98-477C14218035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63E27330-8793-48AB-99AB-A62B2EBFEA49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>rule_type</t>
   </si>
@@ -56,13 +56,25 @@
   </si>
   <si>
     <t>Content.BodyText</t>
+  </si>
+  <si>
+    <t>SANITIZE_HTML</t>
+  </si>
+  <si>
+    <t>Content.Title</t>
+  </si>
+  <si>
+    <t>Attachments[].URL</t>
+  </si>
+  <si>
+    <t>URLs[].URL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -72,6 +84,10 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="3">
@@ -99,13 +115,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -319,7 +341,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="2" width="28" customWidth="1"/>
@@ -362,24 +384,54 @@
       <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
+      <c r="A3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="3"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" t="s">
+      <c r="A4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B6" t="s">
         <v>10</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D6" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: integrate enhanced media summarization into post-normalization
</commit_message>
<xml_diff>
--- a/data/rules/mediaPostNormalization.xlsx
+++ b/data/rules/mediaPostNormalization.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63E27330-8793-48AB-99AB-A62B2EBFEA49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DDC93DE-C833-4D2C-A78D-425394CBC86F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2160" yWindow="1610" windowWidth="13550" windowHeight="9670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
   <si>
     <t>rule_type</t>
   </si>
@@ -68,6 +68,12 @@
   </si>
   <si>
     <t>URLs[].URL</t>
+  </si>
+  <si>
+    <t>GENERATE_MEDIA_SUMMARY</t>
+  </si>
+  <si>
+    <t>Content.Summary</t>
   </si>
 </sst>
 </file>
@@ -341,7 +347,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="2" width="28" customWidth="1"/>
@@ -434,6 +440,17 @@
         <v>13</v>
       </c>
     </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>